<commit_message>
sync: envy · 2026-09-19 19:47:24
</commit_message>
<xml_diff>
--- a/fase_1/salida/tabla_price.xlsx
+++ b/fase_1/salida/tabla_price.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="PS" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="PS" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -223,13 +223,188 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1f497d"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="eeece1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4f81bd"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="c0504d"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9bbb59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064a2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4bacc6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="f79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ff"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:J1048576"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.89"/>
@@ -272,6 +447,336 @@
         <v>9</v>
       </c>
     </row>
+    <row r="1048247" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048248" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048249" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048250" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048251" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048252" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048253" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048254" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048255" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048256" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048257" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048258" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048259" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048260" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048261" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048262" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048263" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048264" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048265" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048266" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048267" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048268" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048269" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048270" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048271" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048272" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048273" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048274" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048275" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048276" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048277" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048278" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048279" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048280" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048281" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048282" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048283" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048284" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048285" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048286" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048287" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048288" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048289" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048290" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048291" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048292" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048293" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048294" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048295" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048296" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048297" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048298" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048299" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048300" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048301" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048302" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048303" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048304" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048305" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048306" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048307" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048308" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048309" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048310" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048311" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048312" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048313" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048314" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048315" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048316" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048317" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048318" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048319" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048320" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048321" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048322" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048323" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048324" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048325" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048326" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048327" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048328" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048329" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048330" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048331" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048332" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048333" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048334" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048335" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048336" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048337" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048338" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048339" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048340" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048341" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048342" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048343" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048344" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048345" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048346" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048347" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048348" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048349" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048350" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048351" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048352" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048353" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048354" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048355" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048356" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048357" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048358" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048359" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048360" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048361" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048362" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048363" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048364" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048365" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048366" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048367" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048368" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048369" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048370" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048371" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048372" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048373" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048374" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048375" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048376" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048377" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048378" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048379" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048380" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048381" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048382" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048383" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048384" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048385" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048386" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048387" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048388" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048389" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048390" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048391" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048392" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048393" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048394" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048395" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048396" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048397" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048398" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048399" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048400" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048401" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048402" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048403" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048404" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048405" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048406" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048407" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048408" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048409" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048410" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048411" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048412" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048413" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048414" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048415" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048416" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048417" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048418" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048419" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048420" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048421" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048422" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048423" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048424" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048425" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048426" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048427" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048428" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048429" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048430" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048431" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048432" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048433" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048434" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048435" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048436" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048437" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048438" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048439" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048440" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048441" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048442" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048443" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048444" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048445" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048446" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048447" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048448" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048449" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048450" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048451" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048452" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048453" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048454" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048455" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048456" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048457" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048458" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048459" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048460" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048461" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048462" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048463" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048464" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048465" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048466" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048467" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048468" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048469" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048470" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048471" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048472" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048473" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048474" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048475" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048476" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048477" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048478" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048479" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048480" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048481" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048482" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048483" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048484" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048485" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048486" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048487" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048488" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048489" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048490" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048491" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048492" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048493" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048494" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048495" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048496" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048497" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048498" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048499" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048500" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048501" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048502" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048503" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048504" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048505" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048506" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048507" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048508" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048509" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048510" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048511" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048512" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048513" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048514" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048515" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048516" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048517" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048518" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048519" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048520" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048521" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048522" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048523" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048524" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048525" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048526" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048527" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048528" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048529" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048530" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048531" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048532" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048533" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048534" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048535" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048536" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048537" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048538" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048539" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048540" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048541" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048542" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048543" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048544" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048545" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048546" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048547" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048548" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048549" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048550" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048551" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048552" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>